<commit_message>
lf10: add S37 + AI B-roll 01-10, S37 script/card wording to AEC, asset list + AI prompt status, PASTE_BRIEF.md
</commit_message>
<xml_diff>
--- a/longform/lf10-kingmaker/assets-list/lf10_Asset_List.xlsx
+++ b/longform/lf10-kingmaker/assets-list/lf10_Asset_List.xlsx
@@ -3735,7 +3735,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1920x1080 headless-Chrome screenshot 19 Oct 2026; + _tall.png for scroll. PAGE SAYS NEW SCHEME COMMENCES 1 JANUARY 2027 (contradicts VO "first of July 2026")</t>
+          <t>1920x1080 headless-Chrome screenshot 19 Oct 2026; + _tall.png for scroll. page: changes from 1 July 2026, new scheme/caps from 1 January 2027 (matches updated S37 VO)</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Parliament passes bill. ParlView: not downloaded (APH Conditions 5.12: fair and accurate reports only, balanced, no digital manipulation, no party/commercial advertising; AUSParliamentLive needs written permission; lf03/lf05/lf09 precedent FREE SWAP). Fallback: DOC_aec_fadreform_2026 + BR_STOCK_parliament_house_canberra</t>
+          <t>Parliament passes bill. ParlView: not downloaded (APH Conditions 5.12: fair and accurate reports only, balanced, no digital manipulation, no party/commercial advertising; AUSParliamentLive needs written permission; lf03/lf05/lf09 precedent FREE SWAP). Fallback: DOC_aec_fadreform_2026 + BR_STOCK_parliament_house_canberra; card: CHANGES FROM 1 JULY 2026 / NATIONAL CAPS FROM 1 JANUARY 2027 / Source: AEC</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>broll/BR_AI_01_driveway_dusk.mp4 (to generate)</t>
+          <t>broll/BR_AI_01_driveway_dusk.mp4</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6502,12 +6502,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>broll/BR_AI_02_ballot_into_box.mp4 (to generate)</t>
+          <t>broll/BR_AI_02_ballot_into_box.mp4</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -6544,12 +6544,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>broll/BR_AI_03_corridor_door_night.mp4 (to generate)</t>
+          <t>broll/BR_AI_03_corridor_door_night.mp4</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6586,12 +6586,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>broll/BR_AI_04_newspaper_doorstep.mp4 (to generate)</t>
+          <t>broll/BR_AI_04_newspaper_doorstep.mp4</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -6628,12 +6628,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>broll/BR_AI_05_newspaper_train_seat.mp4 (to generate)</t>
+          <t>broll/BR_AI_05_newspaper_train_seat.mp4</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6670,12 +6670,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>broll/BR_AI_06_boardroom_empty_chair.mp4 (to generate)</t>
+          <t>broll/BR_AI_06_boardroom_empty_chair.mp4</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -6712,12 +6712,12 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>broll/BR_AI_07_letterbox_flyers.mp4 (to generate)</t>
+          <t>broll/BR_AI_07_letterbox_flyers.mp4</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -6754,12 +6754,12 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>broll/BR_AI_08_phone_glow_dark.mp4 (to generate)</t>
+          <t>broll/BR_AI_08_phone_glow_dark.mp4</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -6796,12 +6796,12 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>broll/BR_AI_09_ballot_count_hands.mp4 (to generate)</t>
+          <t>broll/BR_AI_09_ballot_count_hands.mp4</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -6838,12 +6838,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>broll/BR_AI_10_pencil_marks_ballot.mp4 (to generate)</t>
+          <t>broll/BR_AI_10_pencil_marks_ballot.mp4</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -6880,12 +6880,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>AI-PROMPT</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>prompt in broll/AI_PROMPTS.tsv; label "Dramatised reconstruction"</t>
+          <t>generated 19 Oct 2026; 1280x720, 10 s, has an audio track (mute); Grok watermark bottom-right: crop/cover; prompt in broll/AI_PROMPTS.tsv; first AI clip used gets "Dramatised reconstruction"</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IMG_whitlam_headshot, IMG_whitlam_after_dismissal_1975, IMG_kerr_governor_general, IMG_whitlam_lodge_1974, MUS_01_tense_pulse, SFX_clock_ticks, SFX_drone_low, SFX_bass_impact, BR_AI_01_driveway_dusk (AI-PROMPT), BR_AI_02_ballot_into_box (AI-PROMPT)</t>
+          <t>IMG_whitlam_headshot, IMG_whitlam_after_dismissal_1975, IMG_kerr_governor_general, IMG_whitlam_lodge_1974, MUS_01_tense_pulse, SFX_clock_ticks, SFX_drone_low, SFX_bass_impact, BR_AI_01_driveway_dusk, BR_AI_02_ballot_into_box</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6947,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IMG_parliament_house_flag, IMG_parliament_house_blue_hour, BR_STOCK_parliament_house_canberra, BR_STOCK_printing_press, BR_STOCK_digital_screens, BR_AI_news_desk, BR_AI_strategy_room_whiteboard, MUS_01_tense_pulse, SFX_drone_low, SFX_press_machinery_hum, BR_STOCK_haul_trucks_slowmo (MISSING), BR_AI_03_corridor_door_night (AI-PROMPT)</t>
+          <t>IMG_parliament_house_flag, IMG_parliament_house_blue_hour, BR_STOCK_parliament_house_canberra, BR_STOCK_printing_press, BR_STOCK_digital_screens, BR_AI_news_desk, BR_AI_strategy_room_whiteboard, MUS_01_tense_pulse, SFX_drone_low, SFX_press_machinery_hum, BR_STOCK_haul_trucks_slowmo (MISSING), BR_AI_03_corridor_door_night</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7007,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IMG_rudd_2007, IMG_house_of_reps_chamber, BR_STOCK_newspaper_flipping_pov, BR_STOCK_laptop_typing, MUS_02_investigative, PV03_pm_dispatch_box (MISSING), BR_AI_04_newspaper_doorstep (AI-PROMPT)</t>
+          <t>IMG_rudd_2007, IMG_house_of_reps_chamber, BR_STOCK_newspaper_flipping_pov, BR_STOCK_laptop_typing, MUS_02_investigative, PV03_pm_dispatch_box (MISSING), BR_AI_04_newspaper_doorstep</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IMG_murdoch_2015, IMG_lachlan_murdoch_2018, BR_STOCK_phone_scrolling, MUS_02_investigative, BR_AI_05_newspaper_train_seat (AI-PROMPT)</t>
+          <t>IMG_murdoch_2015, IMG_lachlan_murdoch_2018, BR_STOCK_phone_scrolling, MUS_02_investigative, BR_AI_05_newspaper_train_seat</t>
         </is>
       </c>
     </row>
@@ -7091,7 +7091,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MUS_07_retro_synth, BR_AI_06_boardroom_empty_chair (AI-PROMPT)</t>
+          <t>MUS_07_retro_synth, BR_AI_06_boardroom_empty_chair</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7151,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MUS_08_industrial_percussion, BR_STOCK_highway_billboards (MISSING), BR_AI_07_letterbox_flyers (AI-PROMPT)</t>
+          <t>MUS_08_industrial_percussion, BR_STOCK_highway_billboards (MISSING), BR_AI_07_letterbox_flyers</t>
         </is>
       </c>
     </row>
@@ -7175,7 +7175,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MUS_03_archival, BR_AI_03_corridor_door_night (AI-PROMPT)</t>
+          <t>MUS_03_archival, BR_AI_03_corridor_door_night</t>
         </is>
       </c>
     </row>
@@ -7199,7 +7199,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BR_STOCK_canberra_sunset_sky, MUS_03_archival, BR_AI_08_phone_glow_dark (AI-PROMPT)</t>
+          <t>BR_STOCK_canberra_sunset_sky, MUS_03_archival, BR_AI_08_phone_glow_dark</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7259,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MUS_09_playful_plucks, BR_AI_09_ballot_count_hands (AI-PROMPT)</t>
+          <t>MUS_09_playful_plucks, BR_AI_09_ballot_count_hands</t>
         </is>
       </c>
     </row>
@@ -7427,7 +7427,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IMG_whitlam_headshot, IMG_whitlam_after_dismissal_1975, IMG_dismissal_demonstration_1975, IMG_fraser_1974, IMG_fraser_1977, IMG_whitlam_lodge_1974, MUS_06_tense_resolve, BR_AI_02_ballot_into_box (AI-PROMPT)</t>
+          <t>IMG_whitlam_headshot, IMG_whitlam_after_dismissal_1975, IMG_dismissal_demonstration_1975, IMG_fraser_1974, IMG_fraser_1977, IMG_whitlam_lodge_1974, MUS_06_tense_resolve, BR_AI_02_ballot_into_box</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MUS_06_tense_resolve, SFX_pencil_writing, BR_AI_10_pencil_marks_ballot (AI-PROMPT)</t>
+          <t>MUS_06_tense_resolve, SFX_pencil_writing, BR_AI_10_pencil_marks_ballot</t>
         </is>
       </c>
     </row>

</xml_diff>